<commit_message>
Update Metaculus median (scheduled)
</commit_message>
<xml_diff>
--- a/data/metaculus_shor_rsa_median.xlsx
+++ b/data/metaculus_shor_rsa_median.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,6 +511,14 @@
         <v>48994</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>46054</v>
+      </c>
+      <c r="B12" s="1" t="n">
+        <v>48994</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>